<commit_message>
Reset HR templates to blank forms for public repo
</commit_message>
<xml_diff>
--- a/templates/Claim Statement-2026.xlsx
+++ b/templates/Claim Statement-2026.xlsx
@@ -927,11 +927,7 @@
         </is>
       </c>
       <c r="B4" s="53" t="n"/>
-      <c r="C4" s="56" t="inlineStr">
-        <is>
-          <t>Saswat Suman Mishra</t>
-        </is>
-      </c>
+      <c r="C4" s="56" t="n"/>
       <c r="D4" s="57" t="n"/>
       <c r="E4" s="58" t="n"/>
     </row>
@@ -942,9 +938,7 @@
         </is>
       </c>
       <c r="B5" s="53" t="n"/>
-      <c r="C5" s="59" t="n">
-        <v>75</v>
-      </c>
+      <c r="C5" s="59" t="n"/>
       <c r="D5" s="53" t="n"/>
       <c r="E5" s="54" t="n"/>
       <c r="F5" s="10" t="n"/>
@@ -1196,7 +1190,7 @@
     <row r="35" ht="12.75" customHeight="1" s="51">
       <c r="A35" s="69" t="inlineStr">
         <is>
-          <t>Employee Signature : Saswat Suman Mishra</t>
+          <t>Employee Signature :</t>
         </is>
       </c>
       <c r="B35" s="70" t="n"/>
@@ -2221,7 +2215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G109"/>
+  <dimension ref="A2:G38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.43" customWidth="1" style="51" min="1" max="1"/>
@@ -2262,11 +2256,7 @@
         </is>
       </c>
       <c r="B4" s="53" t="n"/>
-      <c r="C4" s="56" t="inlineStr">
-        <is>
-          <t>Saswat Suman Mishra</t>
-        </is>
-      </c>
+      <c r="C4" s="56" t="n"/>
       <c r="D4" s="57" t="n"/>
       <c r="E4" s="58" t="n"/>
     </row>
@@ -2277,9 +2267,7 @@
         </is>
       </c>
       <c r="B5" s="53" t="n"/>
-      <c r="C5" s="59" t="n">
-        <v>75</v>
-      </c>
+      <c r="C5" s="59" t="n"/>
       <c r="D5" s="53" t="n"/>
       <c r="E5" s="54" t="n"/>
       <c r="F5" s="10" t="n"/>
@@ -2319,2073 +2307,317 @@
       </c>
     </row>
     <row r="8" ht="13.5" customHeight="1" s="51">
-      <c r="A8" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="22" t="n">
-        <v>46124</v>
-      </c>
-      <c r="C8" s="21" t="inlineStr">
-        <is>
-          <t>ba6c48e8-f0f6-49c6-bbf4-3b73e9edbfce</t>
-        </is>
-      </c>
-      <c r="D8" s="21" t="n">
-        <v>839.02</v>
-      </c>
-      <c r="E8" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A8" s="21" t="n"/>
+      <c r="B8" s="22" t="n"/>
+      <c r="C8" s="21" t="n"/>
+      <c r="D8" s="21" t="n"/>
+      <c r="E8" s="21" t="n"/>
     </row>
     <row r="9" ht="13.5" customHeight="1" s="51">
-      <c r="A9" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="22" t="n">
-        <v>46124</v>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>fcee8b51-aae9-4652-891c-e8a89cdd2d2a</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="n">
-        <v>177.7</v>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A9" s="21" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
     </row>
     <row r="10" ht="13.5" customHeight="1" s="51">
-      <c r="A10" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="22" t="n">
-        <v>46125</v>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>1ca35363-6499-4fc1-91ba-6d1515dc25e8</t>
-        </is>
-      </c>
-      <c r="D10" s="21" t="n">
-        <v>67.63</v>
-      </c>
-      <c r="E10" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A10" s="21" t="n"/>
+      <c r="B10" s="22" t="n"/>
+      <c r="C10" s="21" t="n"/>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
     </row>
     <row r="11" ht="13.5" customHeight="1" s="51">
-      <c r="A11" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="22" t="n">
-        <v>46125</v>
-      </c>
-      <c r="C11" s="21" t="inlineStr">
-        <is>
-          <t>26384ebe-2f4e-4816-bb20-fc005357892c</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="n">
-        <v>60.66</v>
-      </c>
-      <c r="E11" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A11" s="21" t="n"/>
+      <c r="B11" s="22" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
     </row>
     <row r="12" ht="13.5" customHeight="1" s="51">
-      <c r="A12" s="21" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="22" t="n">
-        <v>46126</v>
-      </c>
-      <c r="C12" s="21" t="inlineStr">
-        <is>
-          <t>0849cea9-f393-4ef0-b042-50f50c3e5c7c</t>
-        </is>
-      </c>
-      <c r="D12" s="21" t="n">
-        <v>56.03</v>
-      </c>
-      <c r="E12" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A12" s="21" t="n"/>
+      <c r="B12" s="22" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
     </row>
     <row r="13" ht="13.5" customHeight="1" s="51">
-      <c r="A13" s="21" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="22" t="n">
-        <v>46126</v>
-      </c>
-      <c r="C13" s="21" t="inlineStr">
-        <is>
-          <t>75398a89-2461-4db4-bb2d-eedb8032fded</t>
-        </is>
-      </c>
-      <c r="D13" s="21" t="n">
-        <v>62.86</v>
-      </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A13" s="21" t="n"/>
+      <c r="B13" s="22" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
     </row>
     <row r="14" ht="13.5" customHeight="1" s="51">
-      <c r="A14" s="21" t="n">
-        <v>7</v>
-      </c>
-      <c r="B14" s="22" t="n">
-        <v>46127</v>
-      </c>
-      <c r="C14" s="21" t="inlineStr">
-        <is>
-          <t>013e1aff-9b0d-4b8b-8f66-b80c8e1ff929</t>
-        </is>
-      </c>
-      <c r="D14" s="21" t="n">
-        <v>62.94</v>
-      </c>
-      <c r="E14" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A14" s="21" t="n"/>
+      <c r="B14" s="22" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
     </row>
     <row r="15" ht="13.5" customHeight="1" s="51">
-      <c r="A15" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="B15" s="22" t="n">
-        <v>46127</v>
-      </c>
-      <c r="C15" s="21" t="inlineStr">
-        <is>
-          <t>501</t>
-        </is>
-      </c>
-      <c r="D15" s="21" t="n">
-        <v>2143.5</v>
-      </c>
-      <c r="E15" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A15" s="21" t="n"/>
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
     </row>
     <row r="16" ht="13.5" customHeight="1" s="51">
-      <c r="A16" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="22" t="n">
-        <v>46127</v>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>d9eaac2a-6341-4d90-a9e9-917e2a3f52e6</t>
-        </is>
-      </c>
-      <c r="D16" s="21" t="n">
-        <v>70.61</v>
-      </c>
-      <c r="E16" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A16" s="21" t="n"/>
+      <c r="B16" s="22" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="21" t="n"/>
     </row>
     <row r="17" ht="13.5" customHeight="1" s="51">
-      <c r="A17" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="B17" s="22" t="n">
-        <v>46128</v>
-      </c>
-      <c r="C17" s="21" t="inlineStr">
-        <is>
-          <t>19bc2ce6-b6c7-46e1-a271-64b87b97b6cc</t>
-        </is>
-      </c>
-      <c r="D17" s="21" t="n">
-        <v>63.19</v>
-      </c>
-      <c r="E17" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A17" s="21" t="n"/>
+      <c r="B17" s="22" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="21" t="n"/>
     </row>
     <row r="18" ht="13.5" customHeight="1" s="51">
-      <c r="A18" s="21" t="n">
-        <v>11</v>
-      </c>
-      <c r="B18" s="22" t="n">
-        <v>46129</v>
-      </c>
-      <c r="C18" s="21" t="inlineStr">
-        <is>
-          <t>721c29d4-83ac-4774-8527-850b3b4588ff</t>
-        </is>
-      </c>
-      <c r="D18" s="21" t="n">
-        <v>65.77</v>
-      </c>
-      <c r="E18" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A18" s="21" t="n"/>
+      <c r="B18" s="22" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="21" t="n"/>
     </row>
     <row r="19" ht="13.5" customHeight="1" s="51">
-      <c r="A19" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="22" t="n">
-        <v>46132</v>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>17364b6d-5379-495e-87bf-f990be1d4716</t>
-        </is>
-      </c>
-      <c r="D19" s="21" t="n">
-        <v>59.1</v>
-      </c>
-      <c r="E19" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A19" s="21" t="n"/>
+      <c r="B19" s="22" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="21" t="n"/>
     </row>
     <row r="20" ht="13.5" customHeight="1" s="51">
-      <c r="A20" s="21" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="22" t="n">
-        <v>46132</v>
-      </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>6d2ad501-fe30-4187-9f74-a227a8a02663</t>
-        </is>
-      </c>
-      <c r="D20" s="21" t="n">
-        <v>75.17</v>
-      </c>
-      <c r="E20" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A20" s="21" t="n"/>
+      <c r="B20" s="22" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="21" t="n"/>
+      <c r="E20" s="21" t="n"/>
     </row>
     <row r="21" ht="13.5" customHeight="1" s="51">
-      <c r="A21" s="21" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="22" t="n">
-        <v>46133</v>
-      </c>
-      <c r="C21" s="21" t="inlineStr">
-        <is>
-          <t>80b9ee87-7613-4bef-b40b-9a51aefce08e</t>
-        </is>
-      </c>
-      <c r="D21" s="21" t="n">
-        <v>70.41</v>
-      </c>
-      <c r="E21" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A21" s="21" t="n"/>
+      <c r="B21" s="22" t="n"/>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="21" t="n"/>
+      <c r="E21" s="21" t="n"/>
     </row>
     <row r="22" ht="13.5" customHeight="1" s="51">
-      <c r="A22" s="21" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="22" t="n">
-        <v>46134</v>
-      </c>
-      <c r="C22" s="21" t="inlineStr">
-        <is>
-          <t>1ca5148d-999f-46b2-a036-8e7444d22fd2</t>
-        </is>
-      </c>
-      <c r="D22" s="21" t="n">
-        <v>71.23999999999999</v>
-      </c>
-      <c r="E22" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A22" s="21" t="n"/>
+      <c r="B22" s="22" t="n"/>
+      <c r="C22" s="21" t="n"/>
+      <c r="D22" s="21" t="n"/>
+      <c r="E22" s="21" t="n"/>
     </row>
     <row r="23" ht="13.5" customHeight="1" s="51">
-      <c r="A23" s="21" t="n">
-        <v>16</v>
-      </c>
-      <c r="B23" s="22" t="n">
-        <v>46134</v>
-      </c>
-      <c r="C23" s="21" t="inlineStr">
-        <is>
-          <t>34b6a4fc-637f-45ba-b222-1a32da84aa2e</t>
-        </is>
-      </c>
-      <c r="D23" s="21" t="n">
-        <v>67.79000000000001</v>
-      </c>
-      <c r="E23" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="22" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
     </row>
     <row r="24" ht="13.5" customHeight="1" s="51">
-      <c r="A24" s="21" t="n">
-        <v>17</v>
-      </c>
-      <c r="B24" s="22" t="n">
-        <v>46135</v>
-      </c>
-      <c r="C24" s="21" t="inlineStr">
-        <is>
-          <t>46790869-95d5-41df-91a6-04f50dfc9c76</t>
-        </is>
-      </c>
-      <c r="D24" s="21" t="n">
-        <v>79.84</v>
-      </c>
-      <c r="E24" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A24" s="21" t="n"/>
+      <c r="B24" s="22" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="21" t="n"/>
       <c r="G24" s="33" t="n"/>
     </row>
     <row r="25" hidden="1" ht="13.5" customHeight="1" s="51">
-      <c r="A25" s="21" t="n">
-        <v>18</v>
-      </c>
-      <c r="B25" s="22" t="n">
-        <v>46135</v>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>ffd2ade2-2dbe-475e-a7d5-895f9887b976</t>
-        </is>
-      </c>
-      <c r="D25" s="21" t="n">
-        <v>55.88</v>
-      </c>
-      <c r="E25" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A25" s="21" t="n"/>
+      <c r="B25" s="22" t="n"/>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="21" t="n"/>
     </row>
     <row r="26" ht="13.5" customHeight="1" s="51">
-      <c r="A26" s="21" t="n">
-        <v>19</v>
-      </c>
-      <c r="B26" s="22" t="n">
-        <v>46136</v>
-      </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>7bf9c25a-aa27-4258-a577-2c66083e19eb</t>
-        </is>
-      </c>
-      <c r="D26" s="21" t="n">
-        <v>74.8</v>
-      </c>
-      <c r="E26" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A26" s="21" t="n"/>
+      <c r="B26" s="22" t="n"/>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="21" t="n"/>
     </row>
     <row r="27" ht="13.5" customHeight="1" s="51">
-      <c r="A27" s="21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B27" s="22" t="n">
-        <v>46137</v>
-      </c>
-      <c r="C27" s="21" t="inlineStr">
-        <is>
-          <t>635480f7-447a-49c3-a411-7993948a7f06</t>
-        </is>
-      </c>
-      <c r="D27" s="21" t="n">
-        <v>56.23</v>
-      </c>
-      <c r="E27" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A27" s="21" t="n"/>
+      <c r="B27" s="22" t="n"/>
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="21" t="n"/>
     </row>
     <row r="28" ht="13.5" customHeight="1" s="51">
-      <c r="A28" s="21" t="n">
-        <v>21</v>
-      </c>
-      <c r="B28" s="22" t="n">
-        <v>46137</v>
-      </c>
-      <c r="C28" s="21" t="inlineStr">
-        <is>
-          <t>89981381-786d-436c-954e-36720066a40e</t>
-        </is>
-      </c>
-      <c r="D28" s="21" t="n">
-        <v>211.71</v>
-      </c>
-      <c r="E28" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A28" s="21" t="n"/>
+      <c r="B28" s="22" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
     </row>
     <row r="29" ht="13.5" customHeight="1" s="51">
-      <c r="A29" s="21" t="n">
-        <v>22</v>
-      </c>
-      <c r="B29" s="22" t="n">
-        <v>46139</v>
-      </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>5dc23c2b-d457-4f8e-a4c2-b22aa0b3b759</t>
-        </is>
-      </c>
-      <c r="D29" s="21" t="n">
-        <v>56.98</v>
-      </c>
-      <c r="E29" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A29" s="21" t="n"/>
+      <c r="B29" s="22" t="n"/>
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="21" t="n"/>
+      <c r="E29" s="21" t="n"/>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="51">
-      <c r="A30" s="21" t="n">
-        <v>23</v>
-      </c>
-      <c r="B30" s="22" t="n">
-        <v>46139</v>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>b21e5cfd-18a3-4be7-b16f-68b14b96152b</t>
-        </is>
-      </c>
-      <c r="D30" s="21" t="n">
-        <v>104.48</v>
-      </c>
-      <c r="E30" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A30" s="21" t="n"/>
+      <c r="B30" s="22" t="n"/>
+      <c r="C30" s="21" t="n"/>
+      <c r="D30" s="21" t="n"/>
+      <c r="E30" s="21" t="n"/>
     </row>
     <row r="31" ht="13.5" customHeight="1" s="51">
-      <c r="A31" s="21" t="n">
-        <v>24</v>
-      </c>
-      <c r="B31" s="22" t="n">
-        <v>46140</v>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>502</t>
-        </is>
-      </c>
-      <c r="D31" s="21" t="n">
-        <v>1800</v>
-      </c>
-      <c r="E31" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A31" s="21" t="n"/>
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="21" t="n"/>
+      <c r="D31" s="21" t="n"/>
+      <c r="E31" s="21" t="n"/>
     </row>
     <row r="32" ht="13.5" customHeight="1" s="51">
-      <c r="A32" s="21" t="n">
-        <v>25</v>
-      </c>
-      <c r="B32" s="22" t="n">
-        <v>46140</v>
-      </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>96802d3c-f908-4a0a-be5c-0656da6f7a12</t>
-        </is>
-      </c>
-      <c r="D32" s="21" t="n">
-        <v>73.38</v>
-      </c>
-      <c r="E32" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="13.5" customHeight="1" s="51">
-      <c r="A33" s="21" t="n">
-        <v>26</v>
-      </c>
-      <c r="B33" s="22" t="n">
-        <v>46140</v>
-      </c>
-      <c r="C33" s="21" t="inlineStr">
-        <is>
-          <t>d1e091fb-7833-4f1f-8487-dca2db8bb8f3</t>
-        </is>
-      </c>
-      <c r="D33" s="21" t="n">
-        <v>67.97</v>
-      </c>
-      <c r="E33" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="13.5" customHeight="1" s="51">
-      <c r="A34" s="21" t="n">
-        <v>27</v>
-      </c>
-      <c r="B34" s="22" t="n">
-        <v>46141</v>
-      </c>
-      <c r="C34" s="21" t="inlineStr">
-        <is>
-          <t>51411a16-ac03-424e-ad00-76f350139dc0</t>
-        </is>
-      </c>
-      <c r="D34" s="21" t="n">
-        <v>75.61</v>
-      </c>
-      <c r="E34" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="13.5" customHeight="1" s="51">
-      <c r="A35" s="21" t="n">
-        <v>28</v>
-      </c>
-      <c r="B35" s="22" t="n">
-        <v>46141</v>
-      </c>
-      <c r="C35" s="21" t="inlineStr">
-        <is>
-          <t>bb724f6c-7768-4e77-b158-1a08a0f94ac4</t>
-        </is>
-      </c>
-      <c r="D35" s="21" t="n">
-        <v>51.84</v>
-      </c>
-      <c r="E35" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="13.5" customHeight="1" s="51">
-      <c r="A36" s="21" t="n">
-        <v>29</v>
-      </c>
-      <c r="B36" s="22" t="n">
-        <v>46141</v>
-      </c>
-      <c r="C36" s="21" t="inlineStr">
-        <is>
-          <t>e41aaca0-66c0-4a3f-9bda-4a3c2f869cf6</t>
-        </is>
-      </c>
-      <c r="D36" s="21" t="n">
-        <v>81.23999999999999</v>
-      </c>
-      <c r="E36" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="13.5" customHeight="1" s="51">
-      <c r="A37" s="21" t="n">
-        <v>30</v>
-      </c>
-      <c r="B37" s="22" t="n">
-        <v>46142</v>
-      </c>
-      <c r="C37" s="21" t="inlineStr">
-        <is>
-          <t>284c0bd4-9259-45b1-8665-0051f7ae4191</t>
-        </is>
-      </c>
-      <c r="D37" s="21" t="n">
-        <v>69.08</v>
-      </c>
-      <c r="E37" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="13.5" customHeight="1" s="51">
-      <c r="A38" s="21" t="n">
-        <v>31</v>
-      </c>
-      <c r="B38" s="22" t="n">
-        <v>46142</v>
-      </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>64941277-3040-4ada-b11a-4a47135d03ea</t>
-        </is>
-      </c>
-      <c r="D38" s="21" t="n">
-        <v>75.90000000000001</v>
-      </c>
-      <c r="E38" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="13.5" customHeight="1" s="51">
-      <c r="A39" s="21" t="n">
-        <v>32</v>
-      </c>
-      <c r="B39" s="22" t="n">
-        <v>46143</v>
-      </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>719b3e38-aa58-4a1b-8140-a77d06cf7514</t>
-        </is>
-      </c>
-      <c r="D39" s="21" t="n">
-        <v>69.33</v>
-      </c>
-      <c r="E39" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="13.5" customHeight="1" s="51">
-      <c r="A40" s="21" t="n">
-        <v>33</v>
-      </c>
-      <c r="B40" s="22" t="n">
-        <v>46143</v>
-      </c>
-      <c r="C40" s="21" t="inlineStr">
-        <is>
-          <t>da215dd8-e74d-4fd8-be67-4434d94c2ef5</t>
-        </is>
-      </c>
-      <c r="D40" s="21" t="n">
-        <v>584.96</v>
-      </c>
-      <c r="E40" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="13.5" customHeight="1" s="51">
-      <c r="A41" s="21" t="n">
-        <v>34</v>
-      </c>
-      <c r="B41" s="22" t="n">
-        <v>46146</v>
-      </c>
-      <c r="C41" s="21" t="inlineStr">
-        <is>
-          <t>213b4a1f-0520-45b1-bad9-23311fb7f227</t>
-        </is>
-      </c>
-      <c r="D41" s="21" t="n">
-        <v>53.88</v>
-      </c>
-      <c r="E41" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="13.5" customHeight="1" s="51">
-      <c r="A42" s="21" t="n">
-        <v>35</v>
-      </c>
-      <c r="B42" s="22" t="n">
-        <v>46146</v>
-      </c>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>32c7fca6-16e3-4342-a1bd-e5dc8ec48474</t>
-        </is>
-      </c>
-      <c r="D42" s="21" t="n">
-        <v>85.44</v>
-      </c>
-      <c r="E42" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="13.5" customHeight="1" s="51">
-      <c r="A43" s="21" t="n">
-        <v>36</v>
-      </c>
-      <c r="B43" s="22" t="n">
-        <v>46147</v>
-      </c>
-      <c r="C43" s="21" t="inlineStr">
-        <is>
-          <t>663737af-9be0-4976-a087-8ba00568f6b9</t>
-        </is>
-      </c>
-      <c r="D43" s="21" t="n">
-        <v>59.24</v>
-      </c>
-      <c r="E43" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="13.5" customHeight="1" s="51">
-      <c r="A44" s="21" t="n">
-        <v>37</v>
-      </c>
-      <c r="B44" s="22" t="n">
-        <v>46147</v>
-      </c>
-      <c r="C44" s="21" t="inlineStr">
-        <is>
-          <t>b5147aca-fec8-4cef-9333-60194b846de5</t>
-        </is>
-      </c>
-      <c r="D44" s="21" t="n">
-        <v>64.64</v>
-      </c>
-      <c r="E44" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="13.5" customHeight="1" s="51">
-      <c r="A45" s="21" t="n">
-        <v>38</v>
-      </c>
-      <c r="B45" s="22" t="n">
-        <v>46148</v>
-      </c>
-      <c r="C45" s="21" t="inlineStr">
-        <is>
-          <t>24ab9ca0-1533-416a-b9d2-be1016afbc9b</t>
-        </is>
-      </c>
-      <c r="D45" s="21" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="E45" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="13.5" customHeight="1" s="51">
-      <c r="A46" s="21" t="n">
-        <v>39</v>
-      </c>
-      <c r="B46" s="22" t="n">
-        <v>46148</v>
-      </c>
-      <c r="C46" s="21" t="inlineStr">
-        <is>
-          <t>35a23efd-c9be-4af4-8de3-1577f64a37d0</t>
-        </is>
-      </c>
-      <c r="D46" s="21" t="n">
-        <v>68.04000000000001</v>
-      </c>
-      <c r="E46" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="13.5" customHeight="1" s="51">
-      <c r="A47" s="21" t="n">
-        <v>40</v>
-      </c>
-      <c r="B47" s="22" t="n">
-        <v>46149</v>
-      </c>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>add335b0-55f5-45ff-90c3-936fad4273c7</t>
-        </is>
-      </c>
-      <c r="D47" s="21" t="n">
-        <v>53.22</v>
-      </c>
-      <c r="E47" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="13.5" customHeight="1" s="51">
-      <c r="A48" s="21" t="n">
-        <v>41</v>
-      </c>
-      <c r="B48" s="22" t="n">
-        <v>46149</v>
-      </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>da0f8700-e314-4bc1-97c2-9a0b05a82d70</t>
-        </is>
-      </c>
-      <c r="D48" s="21" t="n">
-        <v>67.77</v>
-      </c>
-      <c r="E48" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="13.5" customHeight="1" s="51">
-      <c r="A49" s="21" t="n">
-        <v>42</v>
-      </c>
-      <c r="B49" s="22" t="n">
-        <v>46150</v>
-      </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>1c4fa217-e38f-4446-b45a-25db9fd39af0</t>
-        </is>
-      </c>
-      <c r="D49" s="21" t="n">
-        <v>65.23999999999999</v>
-      </c>
-      <c r="E49" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="13.5" customHeight="1" s="51">
-      <c r="A50" s="21" t="n">
-        <v>43</v>
-      </c>
-      <c r="B50" s="22" t="n">
-        <v>46150</v>
-      </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>6ed18bd4-ed9e-4004-8cee-2fe46028dc8f</t>
-        </is>
-      </c>
-      <c r="D50" s="21" t="n">
-        <v>369.32</v>
-      </c>
-      <c r="E50" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="13.5" customHeight="1" s="51">
-      <c r="A51" s="21" t="n">
-        <v>44</v>
-      </c>
-      <c r="B51" s="22" t="n">
-        <v>46152</v>
-      </c>
-      <c r="C51" s="21" t="inlineStr">
-        <is>
-          <t>fe653436-5676-4282-903e-f829304aafbc</t>
-        </is>
-      </c>
-      <c r="D51" s="21" t="n">
-        <v>140.28</v>
-      </c>
-      <c r="E51" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="13.5" customHeight="1" s="51">
-      <c r="A52" s="21" t="n">
-        <v>45</v>
-      </c>
-      <c r="B52" s="22" t="n">
-        <v>46153</v>
-      </c>
-      <c r="C52" s="21" t="inlineStr">
-        <is>
-          <t>44d54594-50e8-405d-be70-26a2d4d963d9</t>
-        </is>
-      </c>
-      <c r="D52" s="21" t="n">
-        <v>55.16</v>
-      </c>
-      <c r="E52" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="13.5" customHeight="1" s="51">
-      <c r="A53" s="21" t="n">
-        <v>46</v>
-      </c>
-      <c r="B53" s="22" t="n">
-        <v>46153</v>
-      </c>
-      <c r="C53" s="21" t="inlineStr">
-        <is>
-          <t>b985ccd5-f233-48a1-8768-ff5e8b6daec0</t>
-        </is>
-      </c>
-      <c r="D53" s="21" t="n">
-        <v>82.68000000000001</v>
-      </c>
-      <c r="E53" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="13.5" customHeight="1" s="51">
-      <c r="A54" s="21" t="n">
-        <v>47</v>
-      </c>
-      <c r="B54" s="22" t="n">
-        <v>46154</v>
-      </c>
-      <c r="C54" s="21" t="inlineStr">
-        <is>
-          <t>503</t>
-        </is>
-      </c>
-      <c r="D54" s="21" t="n">
-        <v>2754.75</v>
-      </c>
-      <c r="E54" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="13.5" customHeight="1" s="51">
-      <c r="A55" s="21" t="n">
-        <v>48</v>
-      </c>
-      <c r="B55" s="22" t="n">
-        <v>46155</v>
-      </c>
-      <c r="C55" s="21" t="inlineStr">
-        <is>
-          <t>2206740d-0087-4cd8-8bd0-d60832cf5955</t>
-        </is>
-      </c>
-      <c r="D55" s="21" t="n">
-        <v>74.26000000000001</v>
-      </c>
-      <c r="E55" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="13.5" customHeight="1" s="51">
-      <c r="A56" s="21" t="n">
-        <v>49</v>
-      </c>
-      <c r="B56" s="22" t="n">
-        <v>46155</v>
-      </c>
-      <c r="C56" s="21" t="inlineStr">
-        <is>
-          <t>f5f56cb5-5bd6-40fb-a906-514f1da09d51</t>
-        </is>
-      </c>
-      <c r="D56" s="21" t="n">
-        <v>64.26000000000001</v>
-      </c>
-      <c r="E56" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="13.5" customHeight="1" s="51">
-      <c r="A57" s="21" t="n">
-        <v>50</v>
-      </c>
-      <c r="B57" s="22" t="n">
-        <v>46156</v>
-      </c>
-      <c r="C57" s="21" t="inlineStr">
-        <is>
-          <t>0db60e43-9bfe-47ed-a62c-b0b02781ef66</t>
-        </is>
-      </c>
-      <c r="D57" s="21" t="n">
-        <v>427.56</v>
-      </c>
-      <c r="E57" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="13.5" customHeight="1" s="51">
-      <c r="A58" s="21" t="n">
-        <v>51</v>
-      </c>
-      <c r="B58" s="22" t="n">
-        <v>46156</v>
-      </c>
-      <c r="C58" s="21" t="inlineStr">
-        <is>
-          <t>8bd11ddf-aff9-4d50-be67-7a0c61007cd9</t>
-        </is>
-      </c>
-      <c r="D58" s="21" t="n">
-        <v>74.26000000000001</v>
-      </c>
-      <c r="E58" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="13.5" customHeight="1" s="51">
-      <c r="A59" s="21" t="n">
-        <v>52</v>
-      </c>
-      <c r="B59" s="22" t="n">
-        <v>46160</v>
-      </c>
-      <c r="C59" s="21" t="inlineStr">
-        <is>
-          <t>10053749</t>
-        </is>
-      </c>
-      <c r="D59" s="21" t="n">
-        <v>2824.6</v>
-      </c>
-      <c r="E59" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="13.5" customHeight="1" s="51">
-      <c r="A60" s="21" t="n">
-        <v>53</v>
-      </c>
-      <c r="B60" s="22" t="n">
-        <v>46160</v>
-      </c>
-      <c r="C60" s="21" t="inlineStr">
-        <is>
-          <t>18d6cf86-d5b9-4df0-8375-acb5da9634b7</t>
-        </is>
-      </c>
-      <c r="D60" s="21" t="n">
-        <v>61.37</v>
-      </c>
-      <c r="E60" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="13.5" customHeight="1" s="51">
-      <c r="A61" s="21" t="n">
-        <v>54</v>
-      </c>
-      <c r="B61" s="22" t="n">
-        <v>46160</v>
-      </c>
-      <c r="C61" s="21" t="inlineStr">
-        <is>
-          <t>f9f7a2e2-46c4-497a-b739-aeea5b8e12c1</t>
-        </is>
-      </c>
-      <c r="D61" s="21" t="n">
-        <v>75.15000000000001</v>
-      </c>
-      <c r="E61" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="13.5" customHeight="1" s="51">
-      <c r="A62" s="21" t="n">
-        <v>55</v>
-      </c>
-      <c r="B62" s="22" t="n">
-        <v>46161</v>
-      </c>
-      <c r="C62" s="21" t="inlineStr">
-        <is>
-          <t>0a8f0763-3e8a-4239-b08e-eee3f752d307</t>
-        </is>
-      </c>
-      <c r="D62" s="21" t="n">
-        <v>67.77</v>
-      </c>
-      <c r="E62" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="13.5" customHeight="1" s="51">
-      <c r="A63" s="21" t="n">
-        <v>56</v>
-      </c>
-      <c r="B63" s="22" t="n">
-        <v>46163</v>
-      </c>
-      <c r="C63" s="21" t="inlineStr">
-        <is>
-          <t>17db7b1e-735c-4f6b-81da-5fe499a258da</t>
-        </is>
-      </c>
-      <c r="D63" s="21" t="n">
-        <v>56.05</v>
-      </c>
-      <c r="E63" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="13.5" customHeight="1" s="51">
-      <c r="A64" s="21" t="n">
-        <v>57</v>
-      </c>
-      <c r="B64" s="22" t="n">
-        <v>46163</v>
-      </c>
-      <c r="C64" s="21" t="inlineStr">
-        <is>
-          <t>66107b60-d536-4d30-8f9b-44b344356554</t>
-        </is>
-      </c>
-      <c r="D64" s="21" t="n">
-        <v>68.04000000000001</v>
-      </c>
-      <c r="E64" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="13.5" customHeight="1" s="51">
-      <c r="A65" s="21" t="n">
-        <v>58</v>
-      </c>
-      <c r="B65" s="22" t="n">
-        <v>46167</v>
-      </c>
-      <c r="C65" s="21" t="inlineStr">
-        <is>
-          <t>35fbeacd-f991-45e4-a561-207a4a36f688</t>
-        </is>
-      </c>
-      <c r="D65" s="21" t="n">
-        <v>63.84</v>
-      </c>
-      <c r="E65" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="13.5" customHeight="1" s="51">
-      <c r="A66" s="21" t="n">
-        <v>59</v>
-      </c>
-      <c r="B66" s="22" t="n">
-        <v>46167</v>
-      </c>
-      <c r="C66" s="21" t="inlineStr">
-        <is>
-          <t>9258d798-5ea7-4b9f-b003-2425f3ddf25f</t>
-        </is>
-      </c>
-      <c r="D66" s="21" t="n">
-        <v>72.15000000000001</v>
-      </c>
-      <c r="E66" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="13.5" customHeight="1" s="51">
-      <c r="A67" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="B67" s="22" t="n">
-        <v>46168</v>
-      </c>
-      <c r="C67" s="21" t="inlineStr">
-        <is>
-          <t>18690a0e-da5d-4f1f-8ae1-2b38e51a5dd0</t>
-        </is>
-      </c>
-      <c r="D67" s="21" t="n">
-        <v>58.52</v>
-      </c>
-      <c r="E67" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="13.5" customHeight="1" s="51">
-      <c r="A68" s="21" t="n">
-        <v>61</v>
-      </c>
-      <c r="B68" s="22" t="n">
-        <v>46168</v>
-      </c>
-      <c r="C68" s="21" t="inlineStr">
-        <is>
-          <t>504</t>
-        </is>
-      </c>
-      <c r="D68" s="21" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E68" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="13.5" customHeight="1" s="51">
-      <c r="A69" s="21" t="n">
-        <v>62</v>
-      </c>
-      <c r="B69" s="22" t="n">
-        <v>46168</v>
-      </c>
-      <c r="C69" s="21" t="inlineStr">
-        <is>
-          <t>533db946-da89-466a-a94c-6633061f6e0f</t>
-        </is>
-      </c>
-      <c r="D69" s="21" t="n">
-        <v>65.04000000000001</v>
-      </c>
-      <c r="E69" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="13.5" customHeight="1" s="51">
-      <c r="A70" s="21" t="n">
-        <v>63</v>
-      </c>
-      <c r="B70" s="22" t="n">
-        <v>46169</v>
-      </c>
-      <c r="C70" s="21" t="inlineStr">
-        <is>
-          <t>13462523-7008-4c1e-93fa-92a65ac89366</t>
-        </is>
-      </c>
-      <c r="D70" s="21" t="n">
-        <v>64.77</v>
-      </c>
-      <c r="E70" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="13.5" customHeight="1" s="51">
-      <c r="A71" s="21" t="n">
-        <v>64</v>
-      </c>
-      <c r="B71" s="22" t="n">
-        <v>46169</v>
-      </c>
-      <c r="C71" s="21" t="inlineStr">
-        <is>
-          <t>6179fea4-8b82-44af-a83d-6ab049fb89c3</t>
-        </is>
-      </c>
-      <c r="D71" s="21" t="n">
-        <v>65.54000000000001</v>
-      </c>
-      <c r="E71" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="13.5" customHeight="1" s="51">
-      <c r="A72" s="21" t="n">
-        <v>65</v>
-      </c>
-      <c r="B72" s="22" t="n">
-        <v>46170</v>
-      </c>
-      <c r="C72" s="21" t="inlineStr">
-        <is>
-          <t>81cbd6af-58ae-4768-8bac-0561a9f962ec</t>
-        </is>
-      </c>
-      <c r="D72" s="21" t="n">
-        <v>55.42</v>
-      </c>
-      <c r="E72" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="13.5" customHeight="1" s="51">
-      <c r="A73" s="21" t="n">
-        <v>66</v>
-      </c>
-      <c r="B73" s="22" t="n">
-        <v>46171</v>
-      </c>
-      <c r="C73" s="21" t="inlineStr">
-        <is>
-          <t>6a2c9642-94aa-4dce-b473-ea5176d5d7a5</t>
-        </is>
-      </c>
-      <c r="D73" s="21" t="n">
-        <v>605.39</v>
-      </c>
-      <c r="E73" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="13.5" customHeight="1" s="51">
-      <c r="A74" s="21" t="n">
-        <v>67</v>
-      </c>
-      <c r="B74" s="22" t="n">
-        <v>46171</v>
-      </c>
-      <c r="C74" s="21" t="inlineStr">
-        <is>
-          <t>86fdb311-7099-4b99-93df-8eadeb72ca9a</t>
-        </is>
-      </c>
-      <c r="D74" s="21" t="n">
-        <v>71.26000000000001</v>
-      </c>
-      <c r="E74" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="13.5" customHeight="1" s="51">
-      <c r="A75" s="21" t="n">
-        <v>68</v>
-      </c>
-      <c r="B75" s="22" t="n">
-        <v>46173</v>
-      </c>
-      <c r="C75" s="21" t="inlineStr">
-        <is>
-          <t>ca589e47-0a80-4e8e-a836-a40445916dbc</t>
-        </is>
-      </c>
-      <c r="D75" s="21" t="n">
-        <v>315.63</v>
-      </c>
-      <c r="E75" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="13.5" customHeight="1" s="51">
-      <c r="A76" s="21" t="n">
-        <v>69</v>
-      </c>
-      <c r="B76" s="22" t="n">
-        <v>46174</v>
-      </c>
-      <c r="C76" s="21" t="inlineStr">
-        <is>
-          <t>2f4b8216-24c3-4acf-b878-a2fb913b3c73</t>
-        </is>
-      </c>
-      <c r="D76" s="21" t="n">
-        <v>79.34999999999999</v>
-      </c>
-      <c r="E76" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="13.5" customHeight="1" s="51">
-      <c r="A77" s="21" t="n">
-        <v>70</v>
-      </c>
-      <c r="B77" s="22" t="n">
-        <v>46174</v>
-      </c>
-      <c r="C77" s="21" t="inlineStr">
-        <is>
-          <t>f306f503-729e-4a8c-9aaf-54b889cd010e</t>
-        </is>
-      </c>
-      <c r="D77" s="21" t="n">
-        <v>57.47</v>
-      </c>
-      <c r="E77" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="13.5" customHeight="1" s="51">
-      <c r="A78" s="21" t="n">
-        <v>71</v>
-      </c>
-      <c r="B78" s="22" t="n">
-        <v>46175</v>
-      </c>
-      <c r="C78" s="21" t="inlineStr">
-        <is>
-          <t>257e8848-e3a2-422b-92f1-2fcf0b5948e5</t>
-        </is>
-      </c>
-      <c r="D78" s="21" t="n">
-        <v>64.78</v>
-      </c>
-      <c r="E78" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="13.5" customHeight="1" s="51">
-      <c r="A79" s="21" t="n">
-        <v>72</v>
-      </c>
-      <c r="B79" s="22" t="n">
-        <v>46175</v>
-      </c>
-      <c r="C79" s="21" t="inlineStr">
-        <is>
-          <t>7e230d73-070f-42d2-89df-c7db1d02f6e6</t>
-        </is>
-      </c>
-      <c r="D79" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="E79" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="13.5" customHeight="1" s="51">
-      <c r="A80" s="21" t="n">
-        <v>73</v>
-      </c>
-      <c r="B80" s="22" t="n">
-        <v>46176</v>
-      </c>
-      <c r="C80" s="21" t="inlineStr">
-        <is>
-          <t>2a2e23a3-9092-4ebf-b7c3-4b5243898188</t>
-        </is>
-      </c>
-      <c r="D80" s="21" t="n">
-        <v>67.72</v>
-      </c>
-      <c r="E80" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="13.5" customHeight="1" s="51">
-      <c r="A81" s="21" t="n">
-        <v>74</v>
-      </c>
-      <c r="B81" s="22" t="n">
-        <v>46176</v>
-      </c>
-      <c r="C81" s="21" t="inlineStr">
-        <is>
-          <t>568ea7f2-b331-439c-bbbb-92840fb35500</t>
-        </is>
-      </c>
-      <c r="D81" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="E81" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="13.5" customHeight="1" s="51">
-      <c r="A82" s="21" t="n">
-        <v>75</v>
-      </c>
-      <c r="B82" s="22" t="n">
-        <v>46177</v>
-      </c>
-      <c r="C82" s="21" t="inlineStr">
-        <is>
-          <t>2363a3eb-ecf4-411d-b65f-2bf3ca3cf624</t>
-        </is>
-      </c>
-      <c r="D82" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="E82" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="13.5" customHeight="1" s="51">
-      <c r="A83" s="21" t="n">
-        <v>76</v>
-      </c>
-      <c r="B83" s="22" t="n">
-        <v>46177</v>
-      </c>
-      <c r="C83" s="21" t="inlineStr">
-        <is>
-          <t>7d7c1cd3-3155-482e-9077-38b6f1addc4d</t>
-        </is>
-      </c>
-      <c r="D83" s="21" t="n">
-        <v>67.73</v>
-      </c>
-      <c r="E83" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="13.5" customHeight="1" s="51">
-      <c r="A84" s="21" t="n">
-        <v>77</v>
-      </c>
-      <c r="B84" s="22" t="n">
-        <v>46178</v>
-      </c>
-      <c r="C84" s="21" t="inlineStr">
-        <is>
-          <t>7104586e-a2ec-4f5f-a137-48703460b2fc</t>
-        </is>
-      </c>
-      <c r="D84" s="21" t="n">
-        <v>70.05</v>
-      </c>
-      <c r="E84" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="13.5" customHeight="1" s="51">
-      <c r="A85" s="21" t="n">
-        <v>78</v>
-      </c>
-      <c r="B85" s="22" t="n">
-        <v>46178</v>
-      </c>
-      <c r="C85" s="21" t="inlineStr">
-        <is>
-          <t>c63cf879-7d35-4b34-bb2b-566f3330ded8</t>
-        </is>
-      </c>
-      <c r="D85" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="E85" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="13.5" customHeight="1" s="51">
-      <c r="A86" s="21" t="n">
-        <v>79</v>
-      </c>
-      <c r="B86" s="22" t="n">
-        <v>46181</v>
-      </c>
-      <c r="C86" s="21" t="inlineStr">
-        <is>
-          <t>76ed7c49-623b-4b9c-b57c-485c566993d3</t>
-        </is>
-      </c>
-      <c r="D86" s="21" t="n">
-        <v>79.92</v>
-      </c>
-      <c r="E86" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="13.5" customHeight="1" s="51">
-      <c r="A87" s="21" t="n">
-        <v>80</v>
-      </c>
-      <c r="B87" s="22" t="n">
-        <v>46181</v>
-      </c>
-      <c r="C87" s="21" t="inlineStr">
-        <is>
-          <t>a62b4a81-f496-4371-b269-210f8e06ae7a</t>
-        </is>
-      </c>
-      <c r="D87" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="E87" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="13.5" customHeight="1" s="51">
-      <c r="A88" s="21" t="n">
-        <v>81</v>
-      </c>
-      <c r="B88" s="22" t="n">
-        <v>46182</v>
-      </c>
-      <c r="C88" s="21" t="inlineStr">
-        <is>
-          <t>b8247029-6796-40ea-a440-ee1fff012ede</t>
-        </is>
-      </c>
-      <c r="D88" s="21" t="n">
-        <v>68.95999999999999</v>
-      </c>
-      <c r="E88" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="13.5" customHeight="1" s="51">
-      <c r="A89" s="21" t="n">
-        <v>82</v>
-      </c>
-      <c r="B89" s="22" t="n">
-        <v>46182</v>
-      </c>
-      <c r="C89" s="21" t="inlineStr">
-        <is>
-          <t>e24399a8-505d-447f-8ae1-cef090bc1bab</t>
-        </is>
-      </c>
-      <c r="D89" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="E89" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="13.5" customHeight="1" s="51">
-      <c r="A90" s="21" t="n">
-        <v>83</v>
-      </c>
-      <c r="B90" s="22" t="n">
-        <v>46183</v>
-      </c>
-      <c r="C90" s="21" t="inlineStr">
-        <is>
-          <t>409a97dc-c9b1-47c5-87f6-908ab9c50130</t>
-        </is>
-      </c>
-      <c r="D90" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="E90" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="13.5" customHeight="1" s="51">
-      <c r="A91" s="21" t="n">
-        <v>84</v>
-      </c>
-      <c r="B91" s="22" t="n">
-        <v>46183</v>
-      </c>
-      <c r="C91" s="21" t="inlineStr">
-        <is>
-          <t>bcf812e0-3eb9-4232-97d4-aead4ca6143b</t>
-        </is>
-      </c>
-      <c r="D91" s="21" t="n">
-        <v>75.87</v>
-      </c>
-      <c r="E91" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="13.5" customHeight="1" s="51">
-      <c r="A92" s="21" t="n">
-        <v>85</v>
-      </c>
-      <c r="B92" s="22" t="n">
-        <v>46184</v>
-      </c>
-      <c r="C92" s="21" t="inlineStr">
-        <is>
-          <t>c400a901-bea9-4108-937d-e543ce504798</t>
-        </is>
-      </c>
-      <c r="D92" s="21" t="n">
-        <v>71.97</v>
-      </c>
-      <c r="E92" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="13.5" customHeight="1" s="51">
-      <c r="A93" s="21" t="n">
-        <v>86</v>
-      </c>
-      <c r="B93" s="22" t="n">
-        <v>46187</v>
-      </c>
-      <c r="C93" s="21" t="inlineStr">
-        <is>
-          <t>505</t>
-        </is>
-      </c>
-      <c r="D93" s="21" t="n">
-        <v>2101.75</v>
-      </c>
-      <c r="E93" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="13.5" customHeight="1" s="51">
-      <c r="A94" s="21" t="n">
-        <v>87</v>
-      </c>
-      <c r="B94" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="C94" s="21" t="inlineStr">
-        <is>
-          <t>0e455da7-6963-488e-b37a-4a7f4eba086d</t>
-        </is>
-      </c>
-      <c r="D94" s="21" t="n">
-        <v>60</v>
-      </c>
-      <c r="E94" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="13.5" customHeight="1" s="51">
-      <c r="A95" s="21" t="n">
-        <v>88</v>
-      </c>
-      <c r="B95" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="C95" s="21" t="inlineStr">
-        <is>
-          <t>ac783923-caf5-41dd-87ef-97fb04ca3677</t>
-        </is>
-      </c>
-      <c r="D95" s="21" t="n">
-        <v>73.76000000000001</v>
-      </c>
-      <c r="E95" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="13.5" customHeight="1" s="51">
-      <c r="A96" s="21" t="n">
-        <v>89</v>
-      </c>
-      <c r="B96" s="22" t="n">
-        <v>46189</v>
-      </c>
-      <c r="C96" s="21" t="inlineStr">
-        <is>
-          <t>4ab5ff66-3379-4a44-9e6e-3870996b31ad</t>
-        </is>
-      </c>
-      <c r="D96" s="21" t="n">
-        <v>72.26000000000001</v>
-      </c>
-      <c r="E96" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="13.5" customHeight="1" s="51">
-      <c r="A97" s="21" t="n">
-        <v>90</v>
-      </c>
-      <c r="B97" s="22" t="n">
-        <v>46189</v>
-      </c>
-      <c r="C97" s="21" t="inlineStr">
-        <is>
-          <t>52d2d97d-ee2f-407a-bcc8-87831b610431</t>
-        </is>
-      </c>
-      <c r="D97" s="21" t="n">
-        <v>84</v>
-      </c>
-      <c r="E97" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="13.5" customHeight="1" s="51">
-      <c r="A98" s="21" t="n">
-        <v>91</v>
-      </c>
-      <c r="B98" s="22" t="n">
-        <v>46190</v>
-      </c>
-      <c r="C98" s="21" t="inlineStr">
-        <is>
-          <t>783d006a-2696-44f7-adfc-fbce3533ce65</t>
-        </is>
-      </c>
-      <c r="D98" s="21" t="n">
-        <v>71.43000000000001</v>
-      </c>
-      <c r="E98" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="13.5" customHeight="1" s="51">
-      <c r="A99" s="21" t="n">
-        <v>92</v>
-      </c>
-      <c r="B99" s="22" t="n">
-        <v>46191</v>
-      </c>
-      <c r="C99" s="21" t="inlineStr">
-        <is>
-          <t>99219c1d-b37d-4f28-a56e-e8f1a38a46cb</t>
-        </is>
-      </c>
-      <c r="D99" s="21" t="n">
-        <v>57</v>
-      </c>
-      <c r="E99" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="13.5" customHeight="1" s="51">
-      <c r="A100" s="21" t="n">
-        <v>93</v>
-      </c>
-      <c r="B100" s="22" t="n">
-        <v>46191</v>
-      </c>
-      <c r="C100" s="21" t="inlineStr">
-        <is>
-          <t>aee739ef-2d7a-488b-9dca-60fd8adaeb49</t>
-        </is>
-      </c>
-      <c r="D100" s="21" t="n">
-        <v>70.84</v>
-      </c>
-      <c r="E100" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="13.5" customHeight="1" s="51">
-      <c r="A101" s="21" t="n">
-        <v>94</v>
-      </c>
-      <c r="B101" s="22" t="n">
-        <v>46192</v>
-      </c>
-      <c r="C101" s="21" t="inlineStr">
-        <is>
-          <t>5c0ad160-8c89-45f9-a069-c6d762a912c7</t>
-        </is>
-      </c>
-      <c r="D101" s="21" t="n">
-        <v>57</v>
-      </c>
-      <c r="E101" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="13.5" customHeight="1" s="51">
-      <c r="A102" s="21" t="n">
-        <v>95</v>
-      </c>
-      <c r="B102" s="22" t="n">
-        <v>46192</v>
-      </c>
-      <c r="C102" s="21" t="inlineStr">
-        <is>
-          <t>f881e31f-107f-4bab-8c9e-d6c6449fe8ae</t>
-        </is>
-      </c>
-      <c r="D102" s="21" t="n">
-        <v>72.58</v>
-      </c>
-      <c r="E102" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="15" customHeight="1" s="51">
-      <c r="A103" s="16" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>Total Amount Payable</t>
         </is>
       </c>
-      <c r="B103" s="53" t="n"/>
-      <c r="C103" s="54" t="n"/>
-      <c r="D103" s="64">
-        <f>SUM(D8:D102)</f>
+      <c r="B32" s="53" t="n"/>
+      <c r="C32" s="54" t="n"/>
+      <c r="D32" s="64">
+        <f>SUM(D8:D31)</f>
         <v/>
       </c>
-      <c r="E103" s="54" t="n"/>
-    </row>
-    <row r="104" ht="15" customHeight="1" s="51">
-      <c r="A104" s="16" t="inlineStr">
+      <c r="E32" s="54" t="n"/>
+    </row>
+    <row r="33" ht="13.5" customHeight="1" s="51">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>Less:- Travel Advance paid</t>
         </is>
       </c>
-      <c r="B104" s="53" t="n"/>
-      <c r="C104" s="54" t="n"/>
-      <c r="D104" s="65" t="n">
+      <c r="B33" s="53" t="n"/>
+      <c r="C33" s="54" t="n"/>
+      <c r="D33" s="65" t="n">
         <v>0</v>
       </c>
-      <c r="E104" s="54" t="n"/>
-    </row>
-    <row r="105" ht="15" customHeight="1" s="51">
-      <c r="A105" s="66" t="inlineStr">
+      <c r="E33" s="54" t="n"/>
+    </row>
+    <row r="34" ht="13.5" customHeight="1" s="51">
+      <c r="A34" s="66" t="inlineStr">
         <is>
           <t>Net Amount payable</t>
         </is>
       </c>
-      <c r="B105" s="60" t="n"/>
-      <c r="C105" s="67" t="n"/>
-      <c r="D105" s="68">
-        <f>D103-D104</f>
+      <c r="B34" s="60" t="n"/>
+      <c r="C34" s="67" t="n"/>
+      <c r="D34" s="68">
+        <f>D32-D33</f>
         <v/>
       </c>
-      <c r="E105" s="67" t="n"/>
-    </row>
-    <row r="106" ht="12.75" customHeight="1" s="51">
-      <c r="A106" s="69" t="inlineStr">
+      <c r="E34" s="67" t="n"/>
+    </row>
+    <row r="35" ht="13.5" customHeight="1" s="51">
+      <c r="A35" s="69" t="inlineStr">
         <is>
-          <t>Employee Signature : Saswat Suman Mishra</t>
+          <t>Employee Signature :</t>
         </is>
       </c>
-      <c r="B106" s="70" t="n"/>
-      <c r="C106" s="71" t="inlineStr">
+      <c r="B35" s="70" t="n"/>
+      <c r="C35" s="71" t="inlineStr">
         <is>
           <t>Team head or Manager Signature</t>
         </is>
       </c>
-      <c r="D106" s="72" t="inlineStr">
+      <c r="D35" s="72" t="inlineStr">
         <is>
           <t>Finance team Signature</t>
         </is>
       </c>
-      <c r="E106" s="67" t="n"/>
-    </row>
-    <row r="107" ht="16.5" customHeight="1" s="51">
-      <c r="A107" s="73" t="n"/>
-      <c r="B107" s="74" t="n"/>
-      <c r="C107" s="75" t="n"/>
-      <c r="D107" s="76" t="n"/>
-      <c r="E107" s="77" t="n"/>
-    </row>
-    <row r="108" ht="11.25" customHeight="1" s="51">
-      <c r="A108" s="48" t="n"/>
-      <c r="C108" s="48" t="n"/>
-      <c r="D108" s="48" t="n"/>
-    </row>
+      <c r="E35" s="67" t="n"/>
+    </row>
+    <row r="36" ht="13.5" customHeight="1" s="51">
+      <c r="A36" s="73" t="n"/>
+      <c r="B36" s="74" t="n"/>
+      <c r="C36" s="75" t="n"/>
+      <c r="D36" s="76" t="n"/>
+      <c r="E36" s="77" t="n"/>
+    </row>
+    <row r="37" ht="13.5" customHeight="1" s="51">
+      <c r="A37" s="48" t="n"/>
+      <c r="C37" s="48" t="n"/>
+      <c r="D37" s="48" t="n"/>
+    </row>
+    <row r="38" ht="13.5" customHeight="1" s="51"/>
+    <row r="39" ht="13.5" customHeight="1" s="51"/>
+    <row r="40" ht="13.5" customHeight="1" s="51"/>
+    <row r="41" ht="13.5" customHeight="1" s="51"/>
+    <row r="42" ht="13.5" customHeight="1" s="51"/>
+    <row r="43" ht="13.5" customHeight="1" s="51"/>
+    <row r="44" ht="13.5" customHeight="1" s="51"/>
+    <row r="45" ht="13.5" customHeight="1" s="51"/>
+    <row r="46" ht="13.5" customHeight="1" s="51"/>
+    <row r="47" ht="13.5" customHeight="1" s="51"/>
+    <row r="48" ht="13.5" customHeight="1" s="51"/>
+    <row r="49" ht="13.5" customHeight="1" s="51"/>
+    <row r="50" ht="13.5" customHeight="1" s="51"/>
+    <row r="51" ht="13.5" customHeight="1" s="51"/>
+    <row r="52" ht="13.5" customHeight="1" s="51"/>
+    <row r="53" ht="13.5" customHeight="1" s="51"/>
+    <row r="54" ht="13.5" customHeight="1" s="51"/>
+    <row r="55" ht="13.5" customHeight="1" s="51"/>
+    <row r="56" ht="13.5" customHeight="1" s="51"/>
+    <row r="57" ht="13.5" customHeight="1" s="51"/>
+    <row r="58" ht="13.5" customHeight="1" s="51"/>
+    <row r="59" ht="13.5" customHeight="1" s="51"/>
+    <row r="60" ht="13.5" customHeight="1" s="51"/>
+    <row r="61" ht="13.5" customHeight="1" s="51"/>
+    <row r="62" ht="13.5" customHeight="1" s="51"/>
+    <row r="63" ht="13.5" customHeight="1" s="51"/>
+    <row r="64" ht="13.5" customHeight="1" s="51"/>
+    <row r="65" ht="13.5" customHeight="1" s="51"/>
+    <row r="66" ht="13.5" customHeight="1" s="51"/>
+    <row r="67" ht="13.5" customHeight="1" s="51"/>
+    <row r="68" ht="13.5" customHeight="1" s="51"/>
+    <row r="69" ht="13.5" customHeight="1" s="51"/>
+    <row r="70" ht="13.5" customHeight="1" s="51"/>
+    <row r="71" ht="13.5" customHeight="1" s="51"/>
+    <row r="72" ht="13.5" customHeight="1" s="51"/>
+    <row r="73" ht="13.5" customHeight="1" s="51"/>
+    <row r="74" ht="13.5" customHeight="1" s="51"/>
+    <row r="75" ht="13.5" customHeight="1" s="51"/>
+    <row r="76" ht="13.5" customHeight="1" s="51"/>
+    <row r="77" ht="13.5" customHeight="1" s="51"/>
+    <row r="78" ht="13.5" customHeight="1" s="51"/>
+    <row r="79" ht="13.5" customHeight="1" s="51"/>
+    <row r="80" ht="13.5" customHeight="1" s="51"/>
+    <row r="81" ht="13.5" customHeight="1" s="51"/>
+    <row r="82" ht="13.5" customHeight="1" s="51"/>
+    <row r="83" ht="13.5" customHeight="1" s="51"/>
+    <row r="84" ht="13.5" customHeight="1" s="51"/>
+    <row r="85" ht="13.5" customHeight="1" s="51"/>
+    <row r="86" ht="13.5" customHeight="1" s="51"/>
+    <row r="87" ht="13.5" customHeight="1" s="51"/>
+    <row r="88" ht="13.5" customHeight="1" s="51"/>
+    <row r="89" ht="13.5" customHeight="1" s="51"/>
+    <row r="90" ht="13.5" customHeight="1" s="51"/>
+    <row r="91" ht="13.5" customHeight="1" s="51"/>
+    <row r="92" ht="13.5" customHeight="1" s="51"/>
+    <row r="93" ht="13.5" customHeight="1" s="51"/>
+    <row r="94" ht="13.5" customHeight="1" s="51"/>
+    <row r="95" ht="13.5" customHeight="1" s="51"/>
+    <row r="96" ht="13.5" customHeight="1" s="51"/>
+    <row r="97" ht="13.5" customHeight="1" s="51"/>
+    <row r="98" ht="13.5" customHeight="1" s="51"/>
+    <row r="99" ht="13.5" customHeight="1" s="51"/>
+    <row r="100" ht="13.5" customHeight="1" s="51"/>
+    <row r="101" ht="13.5" customHeight="1" s="51"/>
+    <row r="102" ht="13.5" customHeight="1" s="51"/>
+    <row r="103" ht="15" customHeight="1" s="51"/>
+    <row r="104" ht="15" customHeight="1" s="51"/>
+    <row r="105" ht="15" customHeight="1" s="51"/>
+    <row r="106" ht="12.75" customHeight="1" s="51"/>
+    <row r="107" ht="16.5" customHeight="1" s="51"/>
+    <row r="108" ht="11.25" customHeight="1" s="51"/>
     <row r="109" ht="11.25" customHeight="1" s="51"/>
     <row r="110" ht="13.5" customHeight="1" s="51"/>
     <row r="111" ht="13.5" customHeight="1" s="51"/>
@@ -5312,7 +3544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G56"/>
+  <dimension ref="A2:G38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.43" customWidth="1" style="51" min="1" max="1"/>
@@ -5354,11 +3586,7 @@
         </is>
       </c>
       <c r="B4" s="53" t="n"/>
-      <c r="C4" s="56" t="inlineStr">
-        <is>
-          <t>Saswat Suman Mishra</t>
-        </is>
-      </c>
+      <c r="C4" s="56" t="n"/>
       <c r="D4" s="57" t="n"/>
       <c r="E4" s="58" t="n"/>
     </row>
@@ -5369,9 +3597,7 @@
         </is>
       </c>
       <c r="B5" s="53" t="n"/>
-      <c r="C5" s="59" t="n">
-        <v>75</v>
-      </c>
+      <c r="C5" s="59" t="n"/>
       <c r="D5" s="53" t="n"/>
       <c r="E5" s="54" t="n"/>
       <c r="F5" s="10" t="n"/>
@@ -5411,889 +3637,264 @@
       </c>
     </row>
     <row r="8" ht="13.5" customHeight="1" s="51">
-      <c r="A8" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="22" t="n">
-        <v>46113</v>
-      </c>
-      <c r="C8" s="21" t="inlineStr">
-        <is>
-          <t>7956003628</t>
-        </is>
-      </c>
-      <c r="D8" s="21" t="n">
-        <v>702.88</v>
-      </c>
-      <c r="E8" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A8" s="21" t="n"/>
+      <c r="B8" s="22" t="n"/>
+      <c r="C8" s="21" t="n"/>
+      <c r="D8" s="21" t="n"/>
+      <c r="E8" s="21" t="n"/>
     </row>
     <row r="9" ht="13.5" customHeight="1" s="51">
-      <c r="A9" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="22" t="n">
-        <v>46120</v>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>7984187920</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="n">
-        <v>973.08</v>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A9" s="21" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
     </row>
     <row r="10" ht="13.5" customHeight="1" s="51">
-      <c r="A10" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="22" t="n">
-        <v>46126</v>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>0034996041400010</t>
-        </is>
-      </c>
-      <c r="D10" s="21" t="n">
-        <v>380.1</v>
-      </c>
-      <c r="E10" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A10" s="21" t="n"/>
+      <c r="B10" s="22" t="n"/>
+      <c r="C10" s="21" t="n"/>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
     </row>
     <row r="11" ht="13.5" customHeight="1" s="51">
-      <c r="A11" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="22" t="n">
-        <v>46131</v>
-      </c>
-      <c r="C11" s="21" t="inlineStr">
-        <is>
-          <t>0780945041900003</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="n">
-        <v>387.41</v>
-      </c>
-      <c r="E11" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A11" s="21" t="n"/>
+      <c r="B11" s="22" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
     </row>
     <row r="12" ht="13.5" customHeight="1" s="51">
-      <c r="A12" s="21" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="22" t="n">
-        <v>46132</v>
-      </c>
-      <c r="C12" s="21" t="inlineStr">
-        <is>
-          <t>1067432042000007</t>
-        </is>
-      </c>
-      <c r="D12" s="21" t="n">
-        <v>362.26</v>
-      </c>
-      <c r="E12" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A12" s="21" t="n"/>
+      <c r="B12" s="22" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
     </row>
     <row r="13" ht="13.5" customHeight="1" s="51">
-      <c r="A13" s="21" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="22" t="n">
-        <v>46132</v>
-      </c>
-      <c r="C13" s="21" t="inlineStr">
-        <is>
-          <t>8016735683</t>
-        </is>
-      </c>
-      <c r="D13" s="21" t="n">
-        <v>185.58</v>
-      </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A13" s="21" t="n"/>
+      <c r="B13" s="22" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
     </row>
     <row r="14" ht="13.5" customHeight="1" s="51">
-      <c r="A14" s="21" t="n">
-        <v>7</v>
-      </c>
-      <c r="B14" s="22" t="n">
-        <v>46133</v>
-      </c>
-      <c r="C14" s="21" t="inlineStr">
-        <is>
-          <t>0434304042100119</t>
-        </is>
-      </c>
-      <c r="D14" s="21" t="n">
-        <v>273</v>
-      </c>
-      <c r="E14" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A14" s="21" t="n"/>
+      <c r="B14" s="22" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
     </row>
     <row r="15" ht="13.5" customHeight="1" s="51">
-      <c r="A15" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="B15" s="22" t="n">
-        <v>46134</v>
-      </c>
-      <c r="C15" s="21" t="inlineStr">
-        <is>
-          <t>8030432974</t>
-        </is>
-      </c>
-      <c r="D15" s="21" t="n">
-        <v>411.52</v>
-      </c>
-      <c r="E15" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A15" s="21" t="n"/>
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
     </row>
     <row r="16" ht="13.5" customHeight="1" s="51">
-      <c r="A16" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="22" t="n">
-        <v>46135</v>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>0780945042300016</t>
-        </is>
-      </c>
-      <c r="D16" s="21" t="n">
-        <v>371.9</v>
-      </c>
-      <c r="E16" s="21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A16" s="21" t="n"/>
+      <c r="B16" s="22" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="21" t="n"/>
     </row>
     <row r="17" ht="13.5" customHeight="1" s="51">
-      <c r="A17" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="B17" s="25" t="n">
-        <v>46138</v>
-      </c>
-      <c r="C17" s="26" t="inlineStr">
-        <is>
-          <t>8046967539</t>
-        </is>
-      </c>
-      <c r="D17" s="27" t="n">
-        <v>663.72</v>
-      </c>
-      <c r="E17" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A17" s="24" t="n"/>
+      <c r="B17" s="25" t="n"/>
+      <c r="C17" s="26" t="n"/>
+      <c r="D17" s="27" t="n"/>
+      <c r="E17" s="28" t="n"/>
     </row>
     <row r="18" ht="13.5" customHeight="1" s="51">
-      <c r="A18" s="24" t="n">
-        <v>11</v>
-      </c>
-      <c r="B18" s="25" t="n">
-        <v>46142</v>
-      </c>
-      <c r="C18" s="26" t="inlineStr">
-        <is>
-          <t>0153731043000038</t>
-        </is>
-      </c>
-      <c r="D18" s="27" t="n">
-        <v>215.25</v>
-      </c>
-      <c r="E18" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A18" s="24" t="n"/>
+      <c r="B18" s="25" t="n"/>
+      <c r="C18" s="26" t="n"/>
+      <c r="D18" s="27" t="n"/>
+      <c r="E18" s="28" t="n"/>
     </row>
     <row r="19" ht="13.5" customHeight="1" s="51">
-      <c r="A19" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="25" t="n">
-        <v>46147</v>
-      </c>
-      <c r="C19" s="26" t="inlineStr">
-        <is>
-          <t>0000655050500233</t>
-        </is>
-      </c>
-      <c r="D19" s="27" t="n">
-        <v>330.75</v>
-      </c>
-      <c r="E19" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A19" s="24" t="n"/>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="28" t="n"/>
     </row>
     <row r="20" ht="13.5" customHeight="1" s="51">
-      <c r="A20" s="24" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="25" t="n">
-        <v>46149</v>
-      </c>
-      <c r="C20" s="26" t="inlineStr">
-        <is>
-          <t>0318155050700031</t>
-        </is>
-      </c>
-      <c r="D20" s="27" t="n">
-        <v>709.8</v>
-      </c>
-      <c r="E20" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A20" s="24" t="n"/>
+      <c r="B20" s="25" t="n"/>
+      <c r="C20" s="26" t="n"/>
+      <c r="D20" s="27" t="n"/>
+      <c r="E20" s="28" t="n"/>
     </row>
     <row r="21" ht="13.5" customHeight="1" s="51">
-      <c r="A21" s="24" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="25" t="n">
-        <v>46152</v>
-      </c>
-      <c r="C21" s="26" t="inlineStr">
-        <is>
-          <t>0654809051001811</t>
-        </is>
-      </c>
-      <c r="D21" s="27" t="n">
-        <v>1369.8</v>
-      </c>
-      <c r="E21" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A21" s="24" t="n"/>
+      <c r="B21" s="25" t="n"/>
+      <c r="C21" s="26" t="n"/>
+      <c r="D21" s="27" t="n"/>
+      <c r="E21" s="28" t="n"/>
     </row>
     <row r="22" ht="13.5" customHeight="1" s="51">
-      <c r="A22" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="25" t="n">
-        <v>46154</v>
-      </c>
-      <c r="C22" s="26" t="inlineStr">
-        <is>
-          <t>0064131051200081</t>
-        </is>
-      </c>
-      <c r="D22" s="27" t="n">
-        <v>434.3</v>
-      </c>
-      <c r="E22" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A22" s="24" t="n"/>
+      <c r="B22" s="25" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="27" t="n"/>
+      <c r="E22" s="28" t="n"/>
     </row>
     <row r="23" ht="13.5" customHeight="1" s="51">
-      <c r="A23" s="24" t="n">
-        <v>16</v>
-      </c>
-      <c r="B23" s="25" t="n">
-        <v>46161</v>
-      </c>
-      <c r="C23" s="26" t="inlineStr">
-        <is>
-          <t>1067432051900004</t>
-        </is>
-      </c>
-      <c r="D23" s="27" t="n">
-        <v>412.87</v>
-      </c>
-      <c r="E23" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A23" s="24" t="n"/>
+      <c r="B23" s="25" t="n"/>
+      <c r="C23" s="26" t="n"/>
+      <c r="D23" s="27" t="n"/>
+      <c r="E23" s="28" t="n"/>
     </row>
     <row r="24" ht="13.5" customHeight="1" s="51">
-      <c r="A24" s="24" t="n">
-        <v>17</v>
-      </c>
-      <c r="B24" s="25" t="n">
-        <v>46162</v>
-      </c>
-      <c r="C24" s="29" t="inlineStr">
-        <is>
-          <t>0728444052000016</t>
-        </is>
-      </c>
-      <c r="D24" s="27" t="n">
-        <v>460.75</v>
-      </c>
-      <c r="E24" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A24" s="24" t="n"/>
+      <c r="B24" s="25" t="n"/>
+      <c r="C24" s="29" t="n"/>
+      <c r="D24" s="27" t="n"/>
+      <c r="E24" s="28" t="n"/>
     </row>
     <row r="25" ht="13.5" customHeight="1" s="51">
-      <c r="A25" s="24" t="n">
-        <v>18</v>
-      </c>
-      <c r="B25" s="25" t="n">
-        <v>46162</v>
-      </c>
-      <c r="C25" s="29" t="inlineStr">
-        <is>
-          <t>0825592052000153</t>
-        </is>
-      </c>
-      <c r="D25" s="27" t="n">
-        <v>176.66</v>
-      </c>
-      <c r="E25" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A25" s="24" t="n"/>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="27" t="n"/>
+      <c r="E25" s="28" t="n"/>
     </row>
     <row r="26" ht="13.5" customHeight="1" s="51">
-      <c r="A26" s="24" t="n">
-        <v>19</v>
-      </c>
-      <c r="B26" s="25" t="n">
-        <v>46163</v>
-      </c>
-      <c r="C26" s="29" t="inlineStr">
-        <is>
-          <t>0318155052100044</t>
-        </is>
-      </c>
-      <c r="D26" s="27" t="n">
-        <v>286.65</v>
-      </c>
-      <c r="E26" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A26" s="24" t="n"/>
+      <c r="B26" s="25" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="27" t="n"/>
+      <c r="E26" s="28" t="n"/>
     </row>
     <row r="27" ht="13.5" customHeight="1" s="51">
-      <c r="A27" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="B27" s="25" t="n">
-        <v>46164</v>
-      </c>
-      <c r="C27" s="29" t="inlineStr">
-        <is>
-          <t>0049704052200089</t>
-        </is>
-      </c>
-      <c r="D27" s="27" t="n">
-        <v>298.2</v>
-      </c>
-      <c r="E27" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A27" s="24" t="n"/>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="27" t="n"/>
+      <c r="E27" s="28" t="n"/>
     </row>
     <row r="28" ht="13.5" customHeight="1" s="51">
-      <c r="A28" s="24" t="n">
-        <v>21</v>
-      </c>
-      <c r="B28" s="25" t="n">
-        <v>46164</v>
-      </c>
-      <c r="C28" s="29" t="inlineStr">
-        <is>
-          <t>1318340052200004</t>
-        </is>
-      </c>
-      <c r="D28" s="27" t="n">
-        <v>386.4</v>
-      </c>
-      <c r="E28" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A28" s="24" t="n"/>
+      <c r="B28" s="25" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="27" t="n"/>
+      <c r="E28" s="28" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="51">
-      <c r="A29" s="30" t="n">
-        <v>22</v>
-      </c>
-      <c r="B29" s="25" t="n">
-        <v>46166</v>
-      </c>
-      <c r="C29" s="31" t="inlineStr">
-        <is>
-          <t>1081813052400002</t>
-        </is>
-      </c>
-      <c r="D29" s="27" t="n">
-        <v>307.65</v>
-      </c>
-      <c r="E29" s="32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A29" s="30" t="n"/>
+      <c r="B29" s="25" t="n"/>
+      <c r="C29" s="31" t="n"/>
+      <c r="D29" s="27" t="n"/>
+      <c r="E29" s="32" t="n"/>
       <c r="G29" s="33" t="n"/>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="51">
-      <c r="A30" s="24" t="n">
-        <v>23</v>
-      </c>
-      <c r="B30" s="25" t="n">
-        <v>46167</v>
-      </c>
-      <c r="C30" s="29" t="inlineStr">
-        <is>
-          <t>1361386052500068</t>
-        </is>
-      </c>
-      <c r="D30" s="27" t="n">
-        <v>324.45</v>
-      </c>
-      <c r="E30" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A30" s="24" t="n"/>
+      <c r="B30" s="25" t="n"/>
+      <c r="C30" s="29" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="28" t="n"/>
     </row>
     <row r="31" ht="13.5" customHeight="1" s="51">
-      <c r="A31" s="24" t="n">
-        <v>24</v>
-      </c>
-      <c r="B31" s="25" t="n">
-        <v>46168</v>
-      </c>
-      <c r="C31" s="29" t="inlineStr">
-        <is>
-          <t>0825592052600168</t>
-        </is>
-      </c>
-      <c r="D31" s="27" t="n">
-        <v>176.66</v>
-      </c>
-      <c r="E31" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="A31" s="24" t="n"/>
+      <c r="B31" s="25" t="n"/>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="27" t="n"/>
+      <c r="E31" s="28" t="n"/>
     </row>
     <row r="32" ht="13.5" customHeight="1" s="51">
-      <c r="A32" s="24" t="n">
-        <v>25</v>
-      </c>
-      <c r="B32" s="25" t="n">
-        <v>46170</v>
-      </c>
-      <c r="C32" s="29" t="inlineStr">
-        <is>
-          <t>0825592052800193</t>
-        </is>
-      </c>
-      <c r="D32" s="27" t="n">
-        <v>176.66</v>
-      </c>
-      <c r="E32" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="13.5" customHeight="1" s="51">
-      <c r="A33" s="24" t="n">
-        <v>26</v>
-      </c>
-      <c r="B33" s="25" t="n">
-        <v>46173</v>
-      </c>
-      <c r="C33" s="29" t="inlineStr">
-        <is>
-          <t>264RFA3N00001560</t>
-        </is>
-      </c>
-      <c r="D33" s="27" t="n">
-        <v>434.7</v>
-      </c>
-      <c r="E33" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="13.5" customHeight="1" s="51">
-      <c r="A34" s="24" t="n">
-        <v>27</v>
-      </c>
-      <c r="B34" s="25" t="n">
-        <v>46174</v>
-      </c>
-      <c r="C34" s="29" t="inlineStr">
-        <is>
-          <t>8185010767</t>
-        </is>
-      </c>
-      <c r="D34" s="27" t="n">
-        <v>462.78</v>
-      </c>
-      <c r="E34" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="13.5" customHeight="1" s="51">
-      <c r="A35" s="24" t="n">
-        <v>28</v>
-      </c>
-      <c r="B35" s="25" t="n">
-        <v>46177</v>
-      </c>
-      <c r="C35" s="29" t="inlineStr">
-        <is>
-          <t>0825592060400138</t>
-        </is>
-      </c>
-      <c r="D35" s="27" t="n">
-        <v>303.45</v>
-      </c>
-      <c r="E35" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="13.5" customHeight="1" s="51">
-      <c r="A36" s="24" t="n">
-        <v>29</v>
-      </c>
-      <c r="B36" s="25" t="n">
-        <v>46179</v>
-      </c>
-      <c r="C36" s="29" t="inlineStr">
-        <is>
-          <t>0780945060600036</t>
-        </is>
-      </c>
-      <c r="D36" s="27" t="n">
-        <v>255.7</v>
-      </c>
-      <c r="E36" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="13.5" customHeight="1" s="51">
-      <c r="A37" s="24" t="n">
-        <v>30</v>
-      </c>
-      <c r="B37" s="25" t="n">
-        <v>46179</v>
-      </c>
-      <c r="C37" s="29" t="inlineStr">
-        <is>
-          <t>8205567359</t>
-        </is>
-      </c>
-      <c r="D37" s="27" t="n">
-        <v>221.28</v>
-      </c>
-      <c r="E37" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="13.5" customHeight="1" s="51">
-      <c r="A38" s="24" t="n">
-        <v>31</v>
-      </c>
-      <c r="B38" s="25" t="n">
-        <v>46180</v>
-      </c>
-      <c r="C38" s="29" t="inlineStr">
-        <is>
-          <t>0731633060700032</t>
-        </is>
-      </c>
-      <c r="D38" s="27" t="n">
-        <v>237.46</v>
-      </c>
-      <c r="E38" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="13.5" customHeight="1" s="51">
-      <c r="A39" s="24" t="n">
-        <v>32</v>
-      </c>
-      <c r="B39" s="25" t="n">
-        <v>46180</v>
-      </c>
-      <c r="C39" s="29" t="inlineStr">
-        <is>
-          <t>8206593265</t>
-        </is>
-      </c>
-      <c r="D39" s="27" t="n">
-        <v>462.78</v>
-      </c>
-      <c r="E39" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="13.5" customHeight="1" s="51">
-      <c r="A40" s="24" t="n">
-        <v>33</v>
-      </c>
-      <c r="B40" s="25" t="n">
-        <v>46181</v>
-      </c>
-      <c r="C40" s="29" t="inlineStr">
-        <is>
-          <t>8207833225</t>
-        </is>
-      </c>
-      <c r="D40" s="27" t="n">
-        <v>521.58</v>
-      </c>
-      <c r="E40" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="13.5" customHeight="1" s="51">
-      <c r="A41" s="24" t="n">
-        <v>34</v>
-      </c>
-      <c r="B41" s="25" t="n">
-        <v>46181</v>
-      </c>
-      <c r="C41" s="29" t="inlineStr">
-        <is>
-          <t>8209728810</t>
-        </is>
-      </c>
-      <c r="D41" s="27" t="n">
-        <v>185.58</v>
-      </c>
-      <c r="E41" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="13.5" customHeight="1" s="51">
-      <c r="A42" s="24" t="n">
-        <v>35</v>
-      </c>
-      <c r="B42" s="25" t="n">
-        <v>46183</v>
-      </c>
-      <c r="C42" s="29" t="inlineStr">
-        <is>
-          <t>26KVTYOO00006984</t>
-        </is>
-      </c>
-      <c r="D42" s="27" t="n">
-        <v>536.1</v>
-      </c>
-      <c r="E42" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="13.5" customHeight="1" s="51">
-      <c r="A43" s="24" t="n">
-        <v>36</v>
-      </c>
-      <c r="B43" s="25" t="n">
-        <v>46187</v>
-      </c>
-      <c r="C43" s="29" t="inlineStr">
-        <is>
-          <t>0654809061400111</t>
-        </is>
-      </c>
-      <c r="D43" s="27" t="n">
-        <v>1786.95</v>
-      </c>
-      <c r="E43" s="28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="13.5" customHeight="1" s="51">
-      <c r="A44" s="24" t="n">
-        <v>37</v>
-      </c>
-      <c r="B44" s="25" t="n"/>
-      <c r="C44" s="29" t="n"/>
-      <c r="D44" s="27" t="n"/>
-      <c r="E44" s="28" t="n"/>
-    </row>
-    <row r="45" ht="13.5" customHeight="1" s="51">
-      <c r="A45" s="24" t="n">
-        <v>38</v>
-      </c>
-      <c r="B45" s="25" t="n"/>
-      <c r="C45" s="29" t="n"/>
-      <c r="D45" s="27" t="n"/>
-      <c r="E45" s="28" t="n"/>
-    </row>
-    <row r="46" ht="13.5" customHeight="1" s="51">
-      <c r="A46" s="24" t="n">
-        <v>39</v>
-      </c>
-      <c r="B46" s="25" t="n"/>
-      <c r="C46" s="29" t="n"/>
-      <c r="D46" s="27" t="n"/>
-      <c r="E46" s="28" t="n"/>
-    </row>
-    <row r="47" ht="13.5" customHeight="1" s="51">
-      <c r="A47" s="24" t="n">
-        <v>40</v>
-      </c>
-      <c r="B47" s="25" t="n"/>
-      <c r="C47" s="29" t="n"/>
-      <c r="D47" s="27" t="n"/>
-      <c r="E47" s="28" t="n"/>
-    </row>
-    <row r="48" ht="13.5" customHeight="1" s="51">
-      <c r="A48" s="24" t="n">
-        <v>41</v>
-      </c>
-      <c r="B48" s="25" t="n"/>
-      <c r="C48" s="29" t="n"/>
-      <c r="D48" s="27" t="n"/>
-      <c r="E48" s="28" t="n"/>
-    </row>
-    <row r="49" ht="15" customHeight="1" s="51">
-      <c r="A49" s="30" t="n">
-        <v>42</v>
-      </c>
-      <c r="B49" s="25" t="n"/>
-      <c r="C49" s="31" t="n"/>
-      <c r="D49" s="27" t="n"/>
-      <c r="E49" s="32" t="n"/>
-      <c r="G49" s="33" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1" s="51">
-      <c r="A50" s="16" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>Total Amount Payable</t>
         </is>
       </c>
-      <c r="B50" s="53" t="n"/>
-      <c r="C50" s="54" t="n"/>
-      <c r="D50" s="64">
-        <f>SUM(D8:D43)</f>
+      <c r="B32" s="53" t="n"/>
+      <c r="C32" s="54" t="n"/>
+      <c r="D32" s="64">
+        <f>SUM(D8:D31)</f>
         <v/>
       </c>
-      <c r="E50" s="54" t="n"/>
-    </row>
-    <row r="51" ht="15" customHeight="1" s="51">
-      <c r="A51" s="16" t="inlineStr">
+      <c r="E32" s="54" t="n"/>
+    </row>
+    <row r="33" ht="13.5" customHeight="1" s="51">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>Less:- Travel Advance paid</t>
         </is>
       </c>
-      <c r="B51" s="53" t="n"/>
-      <c r="C51" s="54" t="n"/>
-      <c r="D51" s="65" t="n">
+      <c r="B33" s="53" t="n"/>
+      <c r="C33" s="54" t="n"/>
+      <c r="D33" s="65" t="n">
         <v>0</v>
       </c>
-      <c r="E51" s="54" t="n"/>
-    </row>
-    <row r="52" ht="15" customHeight="1" s="51">
-      <c r="A52" s="66" t="inlineStr">
+      <c r="E33" s="54" t="n"/>
+    </row>
+    <row r="34" ht="13.5" customHeight="1" s="51">
+      <c r="A34" s="66" t="inlineStr">
         <is>
           <t>Net Amount payable</t>
         </is>
       </c>
-      <c r="B52" s="60" t="n"/>
-      <c r="C52" s="67" t="n"/>
-      <c r="D52" s="68">
-        <f>D50-D51</f>
+      <c r="B34" s="60" t="n"/>
+      <c r="C34" s="67" t="n"/>
+      <c r="D34" s="68">
+        <f>D32-D33</f>
         <v/>
       </c>
-      <c r="E52" s="67" t="n"/>
-    </row>
-    <row r="53" ht="12.75" customHeight="1" s="51">
-      <c r="A53" s="69" t="inlineStr">
+      <c r="E34" s="67" t="n"/>
+    </row>
+    <row r="35" ht="13.5" customHeight="1" s="51">
+      <c r="A35" s="69" t="inlineStr">
         <is>
-          <t>Employee Signature : Saswat Suman Mishra</t>
+          <t>Employee Signature :</t>
         </is>
       </c>
-      <c r="B53" s="70" t="n"/>
-      <c r="C53" s="71" t="inlineStr">
+      <c r="B35" s="70" t="n"/>
+      <c r="C35" s="71" t="inlineStr">
         <is>
           <t>Team head or Manager Signature</t>
         </is>
       </c>
-      <c r="D53" s="72" t="inlineStr">
+      <c r="D35" s="72" t="inlineStr">
         <is>
           <t>Finance team Signature</t>
         </is>
       </c>
-      <c r="E53" s="67" t="n"/>
-    </row>
-    <row r="54" ht="16.5" customHeight="1" s="51">
-      <c r="A54" s="73" t="n"/>
-      <c r="B54" s="74" t="n"/>
-      <c r="C54" s="75" t="n"/>
-      <c r="D54" s="76" t="n"/>
-      <c r="E54" s="77" t="n"/>
-    </row>
-    <row r="55" ht="11.25" customHeight="1" s="51">
-      <c r="A55" s="48" t="n"/>
-      <c r="C55" s="48" t="n"/>
-      <c r="D55" s="48" t="n"/>
-    </row>
+      <c r="E35" s="67" t="n"/>
+    </row>
+    <row r="36" ht="13.5" customHeight="1" s="51">
+      <c r="A36" s="73" t="n"/>
+      <c r="B36" s="74" t="n"/>
+      <c r="C36" s="75" t="n"/>
+      <c r="D36" s="76" t="n"/>
+      <c r="E36" s="77" t="n"/>
+    </row>
+    <row r="37" ht="13.5" customHeight="1" s="51">
+      <c r="A37" s="48" t="n"/>
+      <c r="C37" s="48" t="n"/>
+      <c r="D37" s="48" t="n"/>
+    </row>
+    <row r="38" ht="13.5" customHeight="1" s="51"/>
+    <row r="39" ht="13.5" customHeight="1" s="51"/>
+    <row r="40" ht="13.5" customHeight="1" s="51"/>
+    <row r="41" ht="13.5" customHeight="1" s="51"/>
+    <row r="42" ht="13.5" customHeight="1" s="51"/>
+    <row r="43" ht="13.5" customHeight="1" s="51"/>
+    <row r="44" ht="13.5" customHeight="1" s="51"/>
+    <row r="45" ht="13.5" customHeight="1" s="51"/>
+    <row r="46" ht="13.5" customHeight="1" s="51"/>
+    <row r="47" ht="13.5" customHeight="1" s="51"/>
+    <row r="48" ht="13.5" customHeight="1" s="51"/>
+    <row r="49" ht="15" customHeight="1" s="51"/>
+    <row r="50" ht="15" customHeight="1" s="51"/>
+    <row r="51" ht="15" customHeight="1" s="51"/>
+    <row r="52" ht="15" customHeight="1" s="51"/>
+    <row r="53" ht="12.75" customHeight="1" s="51"/>
+    <row r="54" ht="16.5" customHeight="1" s="51"/>
+    <row r="55" ht="11.25" customHeight="1" s="51"/>
     <row r="56" ht="11.25" customHeight="1" s="51"/>
     <row r="57" ht="13.5" customHeight="1" s="51"/>
     <row r="58" ht="13.5" customHeight="1" s="51"/>

</xml_diff>